<commit_message>
election history: 1 events, 2026-06-02 21:37:52
</commit_message>
<xml_diff>
--- a/election_history.xlsx
+++ b/election_history.xlsx
@@ -52,13 +52,13 @@
     <t>Error</t>
   </si>
   <si>
-    <t>2026-06-02T21:33:13.9620764+05:30</t>
+    <t>2026-06-02T21:37:22.3243742+05:30</t>
   </si>
   <si>
     <t>2026-06-02</t>
   </si>
   <si>
-    <t>21:33:13.962</t>
+    <t>21:37:22.324</t>
   </si>
   <si>
     <t>renewed</t>
@@ -79,7 +79,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-06-02T21:35:49+05:30</t>
+    <t>2026-06-02T21:37:52+05:30</t>
   </si>
   <si>
     <t>Total events</t>

</xml_diff>

<commit_message>
election history: 5 events, 2026-06-02 21:47:54
</commit_message>
<xml_diff>
--- a/election_history.xlsx
+++ b/election_history.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>#</t>
   </si>
@@ -76,10 +76,34 @@
     <t/>
   </si>
   <si>
+    <t>2026-06-02T21:39:54.4939959+05:30</t>
+  </si>
+  <si>
+    <t>21:39:54.493</t>
+  </si>
+  <si>
+    <t>2026-06-02T21:42:23.7298825+05:30</t>
+  </si>
+  <si>
+    <t>21:42:23.729</t>
+  </si>
+  <si>
+    <t>2026-06-02T21:44:53.8544422+05:30</t>
+  </si>
+  <si>
+    <t>21:44:53.854</t>
+  </si>
+  <si>
+    <t>2026-06-02T21:47:23.880142+05:30</t>
+  </si>
+  <si>
+    <t>21:47:23.880</t>
+  </si>
+  <si>
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-06-02T21:38:12+05:30</t>
+    <t>2026-06-02T21:47:53+05:30</t>
   </si>
   <si>
     <t>Total events</t>
@@ -552,18 +576,170 @@
         <v>19</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="4">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="4">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="4">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>